<commit_message>
test(fixtures): regenerate sample_bank__qc.expected.xlsx for new behaviour
The bundled expected workbook is rebuilt from sample_bank.xlsx +
sample_bank.expected_verdicts.json under the new writer so newcomers
opening it see the production-ready Corrected sheet (ALIGNED rows
verbatim, NEEDS_EDITS rows with edits applied) and the qc_changes
column on the original sheet.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sample_bank__qc.expected.xlsx
+++ b/examples/sample_bank__qc.expected.xlsx
@@ -55,14 +55,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFD966"/>
+        <bgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
-        <bgColor rgb="00FFD966"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,16 +78,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -454,8 +460,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -523,6 +532,11 @@
           <t>qc_status</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>qc_changes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -694,6 +708,13 @@
           <t>NEEDS_EDITS</t>
         </is>
       </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTNESS: Marked option3 but option3 has two grammatical errors ('were decided'). Only option2 is the defensibly-correct SVA construction.
+EDITS APPLIED:
+  • correctOption: fixes correctness</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -751,6 +772,13 @@
           <t>NEEDS_EDITS</t>
         </is>
       </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>DIFFICULTY: Marked EASY but the prepositional-phrase-between-subject-and-verb trap trips ~30% of MQCs (Angoff ~70%, MEDIUM-band behaviour). Simplify the stem of option2 to drop the trap and return to EASY-band Angoff.
+EDITS APPLIED:
+  • option2: removes the intervening prepositional phrase so the SVA error is obvious; Angoff returns to ~85% EASY band</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -865,6 +893,13 @@
           <t>NEEDS_EDITS</t>
         </is>
       </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTNESS: Two defensibly-correct options: option2 (simple past) and option3 (present perfect, which native speakers accept with 'yesterday' in casual register). Rewrite option3 to break the tie.
+EDITS APPLIED:
+  • option3: switches the time adverb so present-perfect aligns with the verb form; option2 remains the only correct answer for the marked stem</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -917,9 +952,15 @@
           <t>EASY</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>NEEDS_EDITS</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTNESS: Construct mismatch — item tests arithmetic but is tagged subject='Verbal Ability', topics='Grammar and Sentence Correction'. Cannot align via content edits without rewriting the entire question as a grammar item. Escalate to the author.
+EDITS: none auto-applied — human review required</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1058,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
@@ -1034,24 +1075,24 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>AMBER</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>qc_status cell (Original) · whole row (Corrected)</t>
+          <t>qc_status + qc_changes cells (Original) · whole row (Corrected)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NEEDS_EDITS — apply the edits shown in the Corrected sheet.</t>
+          <t>NEEDS_EDITS — apply the edits shown in the Corrected sheet; qc_changes carries the narrative.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>DARK AMBER</t>
         </is>
@@ -1068,14 +1109,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>qc_status cell (Original) · whole row (Corrected)</t>
+          <t>qc_status + qc_changes cells (Original) · whole row (Corrected)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1085,9 +1126,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>How to use: scan the qc_status column on the original sheet. For each amber or red row, open the same row number on the 'Corrected' sheet — the cells highlighted in dark amber are the ones that changed; non-edited cells in that row are shown for context.</t>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>How to use: scan the qc_status column on the original sheet. For each amber or red row, read the qc_changes cell for the full narrative (correctness issue, difficulty issue, and every edit applied), then open the same row number on the 'Corrected' sheet — the cells highlighted in dark amber are the ones that changed. The Corrected sheet is the production-ready output: ALIGNED rows carry the original content verbatim so you can upload the sheet as-is (drop the fills first if your platform doesn't ignore them).</t>
         </is>
       </c>
     </row>
@@ -1171,32 +1212,112 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Identify the grammatically correct sentence.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;She don't likes coffee in the morning.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;She doesn't like coffee in the morning.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;She doesn't likes coffee in the morning.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;She don't like coffee in the morning.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>option2</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_CHOICE_QUESTION</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Verbal Ability</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Grammar and Sentence Correction</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Which is the most appropriate opening for a first-time business email to a senior client?&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Yo!&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Mr. Sharma,&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Hey Sharma,&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Sup boss,&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>option2</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_CHOICE_QUESTION</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Verbal Ability</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Business Communication</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1226,7 +1347,7 @@
       </c>
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>option2</t>
         </is>
@@ -1263,7 +1384,7 @@
           <t>&lt;p&gt;The team has finished its work on schedule.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>&lt;p&gt;The list were reviewed during the morning call.&lt;/p&gt;</t>
         </is>
@@ -1307,18 +1428,58 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Identify the grammatically incorrect sentence.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Neither the manager nor the analysts have submitted the report.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Neither the analysts nor the manager has submitted the report.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Neither the manager nor the analyst has submitted the report.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Neither the analysts nor the manager have submitted the report.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>option4</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_CHOICE_QUESTION</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Verbal Ability</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Grammar and Sentence Correction</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1336,7 +1497,7 @@
           <t>&lt;p&gt;She completed her work yesterday.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>&lt;p&gt;She has completed her work today.&lt;/p&gt;</t>
         </is>
@@ -1375,72 +1536,112 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>&lt;p&gt;If a train covers 240 km in 4 hours, what is its average speed in km/h?&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>&lt;p&gt;40&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>&lt;p&gt;60&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>&lt;p&gt;80&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>&lt;p&gt;100&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>option2</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>MULTIPLE_CHOICE_QUESTION</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Verbal Ability</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Grammar and Sentence Correction</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>EASY</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Passage: A small team of researchers introduced a new metric for measuring code quality that combined cyclomatic complexity with test coverage. Adoption in industry was limited because most teams already used coverage alone and found the new metric harder to explain to leadership.&lt;br&gt;&lt;br&gt;What is the most likely reason adoption was limited?&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;The new metric was less accurate than existing measures.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;The new metric added explanatory cost without a clearly perceived gain.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;The researchers refused to share the formula publicly.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Coverage alone is already a perfect quality measure.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>option2</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_CHOICE_QUESTION</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Verbal Ability</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Reading Comprehension</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>